<commit_message>
feat(master-docs): synchronize manuscript tables workbook metrics with certified holdout and resilience pipelines (v5.14)
</commit_message>
<xml_diff>
--- a/master-docs/thesis_manuscript_tables.xlsx
+++ b/master-docs/thesis_manuscript_tables.xlsx
@@ -1725,12 +1725,12 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>0.5891</t>
+          <t>0.7120</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>0.7588</t>
+          <t>0.7483</t>
         </is>
       </c>
       <c r="F9" s="19" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="G9" s="19" t="inlineStr">
         <is>
-          <t>148.6</t>
+          <t>142.8</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1750,7 +1750,7 @@
       </c>
       <c r="I9" s="19" t="inlineStr">
         <is>
-          <t>-4.2</t>
+          <t>-8.5</t>
         </is>
       </c>
       <c r="J9" s="10" t="inlineStr">
@@ -1763,7 +1763,7 @@
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Note. Master model benchmark matrix evaluated across 72,053 hourly checkpoint observations in the 2025 prospective holdout across 12 carrier complexes (P267 / image15.png). Target variable: hourly throughput volatility (sigma_TSA,hr).</t>
+          <t>Note. Master model benchmark matrix evaluated across 72,053 hourly checkpoint observations in the 2025 prospective holdout across 12 carrier complexes (P267). Target variable: hourly throughput volatility (sigma_TSA,hr). Fully synchronized with Chapter IV text (P273: Test R² = 0.7483, RMSE = 222.1, MASE = 0.662) and 04_model_execution_2025_holdout.xlsx.</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.680–0.700</t>
         </is>
       </c>
       <c r="H7" s="18" t="inlineStr">
@@ -2028,27 +2028,27 @@
       </c>
       <c r="E9" s="18" t="inlineStr">
         <is>
-          <t>487.2 pax/hr</t>
+          <t>398.2 pax/hr</t>
         </is>
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>512.4 pax/hr</t>
+          <t>412.8 pax/hr</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>468.2 pax/hr</t>
+          <t>318.4 pax/hr</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr">
         <is>
-          <t>284.5 pax/hr</t>
+          <t>254.2 pax/hr</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Model 3 Decisive Winner; cuts shock error by 39% and resolves the Empty Checkpoint Fallacy.</t>
+          <t>Model 3 Decisive Winner; cuts shock error by 35.9% vs Model 1 and resolves the Empty Checkpoint Fallacy.</t>
         </is>
       </c>
     </row>
@@ -2075,27 +2075,27 @@
       </c>
       <c r="E10" s="18" t="inlineStr">
         <is>
-          <t>1.921</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>1.632</t>
+          <t>1.320</t>
         </is>
       </c>
       <c r="G10" s="18" t="inlineStr">
         <is>
-          <t>1.698</t>
+          <t>2.140</t>
         </is>
       </c>
       <c r="H10" s="18" t="inlineStr">
         <is>
-          <t>1.281</t>
+          <t>1.050</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Target Met by Model 3; error degrades only +28% vs +70% for pure ML during shocks.</t>
+          <t>Target Met by Model 3 (Winner); live feedback prevents collapse; pure ML collapses (R = 2.14).</t>
         </is>
       </c>
     </row>
@@ -2122,17 +2122,17 @@
       </c>
       <c r="E11" s="18" t="inlineStr">
         <is>
-          <t>18.4 hours</t>
+          <t>8.4 hours</t>
         </is>
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>8.2 hours</t>
+          <t>7.8 hours</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>6.5 hours</t>
+          <t>5.4 hours</t>
         </is>
       </c>
       <c r="H11" s="18" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Target Met by Model 3; real-time recursive loop clears queue backlogs in &lt; 3 hours.</t>
+          <t>Target Met by Model 3 (Winner); real-time recursive loop clears queue backlogs in &lt; 3 hours.</t>
         </is>
       </c>
     </row>
@@ -2184,12 +2184,12 @@
       </c>
       <c r="H12" s="18" t="inlineStr">
         <is>
-          <t>-3.8 pax/hr</t>
+          <t>-14.8 pax/hr</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Target Met by Model 3; prevents structural under-prediction during post-shock surge.</t>
+          <t>Target Met by Model 3; caps bias shift at -14.8 pax/hr, preventing structural under-prediction.</t>
         </is>
       </c>
     </row>
@@ -2248,42 +2248,42 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Relative Transfer Degradation</t>
+          <t>Relative Transfer Ratio (RTR)</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Percentage increase in error when transferred from source to target facilities</t>
+          <t>Ratio of transfer RMSE to in-sample RMSE (EWR -&gt; LGA)</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>ΔMASE ≤ 10.0%</t>
+          <t>RTR ≈ 1.00</t>
         </is>
       </c>
       <c r="E14" s="18" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="F14" s="18" t="inlineStr">
         <is>
-          <t>+4.2%</t>
+          <t>1.04</t>
         </is>
       </c>
       <c r="G14" s="18" t="inlineStr">
         <is>
-          <t>+26.4%</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="H14" s="18" t="inlineStr">
         <is>
-          <t>+42.3%</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Target Met by Model 1; highly portable; pure ML overfits source facility topology.</t>
+          <t>Model 1 Decisive Winner (RTR = 1.04); Model 3 fails target (RTR = 1.19) due to facility overfitting.</t>
         </is>
       </c>
     </row>
@@ -2295,97 +2295,191 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>Relative Transfer Degradation</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Percentage increase in error when transferred from source to target facilities</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>ΔRMSE ≤ 10.0%</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>+4.2%</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>+7.9%</t>
+        </is>
+      </c>
+      <c r="H15" s="18" t="inlineStr">
+        <is>
+          <t>+19.0%</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Target Met by Model 1; highly portable; pure ML and hybrids experience higher transfer penalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 3: Generalizability</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Change in MASE on Transfer</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Absolute change in MASE during zero-shot transfer</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>ΔMASE ≤ 10.0%</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>+4.0% (+0.038)</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>+8.3% (+0.065)</t>
+        </is>
+      </c>
+      <c r="H16" s="18" t="inlineStr">
+        <is>
+          <t>+21.5% (+0.142)</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Model 1 passes target (+4.0%); Model 3 decisively fails (+21.5%) due to decision tree terminal overfitting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 3: Generalizability</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
           <t>Zero-Retraining Portability</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Operational ranking of deployment feasibility across new terminal complexes</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>Highest Portability</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>Rank 4</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Rank 1 (Immediate Zero-Shot)</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G17" s="18" t="inlineStr">
         <is>
           <t>Rank 3 (Requires Retraining)</t>
         </is>
       </c>
-      <c r="H15" s="18" t="inlineStr">
+      <c r="H17" s="18" t="inlineStr">
         <is>
           <t>Rank 2 (Needs Live Sensors)</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Proves Deterministic schedules provide optimal plug-and-play airport portability.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="11" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>Synthesis Finding</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Hypothesis 1 Confirmation</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>Multi-dimensional Pareto dominance audit</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>Multi-dimensional Pareto dominance audit across Robustness, Resilience, Generalizability</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Asymmetric Pareto Dominance</t>
         </is>
       </c>
-      <c r="E16" s="20" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="F16" s="20" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>Winner: Generalizability</t>
         </is>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G18" s="20" t="inlineStr">
         <is>
           <t>Pareto: Routine Efficiency</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>Winner: Shock Resilience</t>
         </is>
       </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="I18" s="11" t="inlineStr">
         <is>
           <t>Hypothesis 1 CONFIRMED: No single modeling paradigm wins across all operational dimensions.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="8" customHeight="1"/>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Note. Master multi-pillar hypothesis evaluation matrix confirming Asymmetric Trade-Offs (H1) across Robustness, Resilience, and Generalizability (P279 / image16.png).</t>
+    <row r="19" ht="8" customHeight="1"/>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Note. Master multi-pillar hypothesis evaluation matrix confirming Asymmetric Trade-Offs (H1) across Robustness, Resilience, and Generalizability (P279). Fully synchronized with Chapter IV prose (P284), Chapter V tables (Table 5.1, 5.2, 5.3), and 05_robustness_resilience_generalizability.xlsx.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(master-docs): add for-deck tab to thesis_manuscript_tables.xlsx with certified Slide 22 metrics (v5.22)
</commit_message>
<xml_diff>
--- a/master-docs/thesis_manuscript_tables.xlsx
+++ b/master-docs/thesis_manuscript_tables.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_5_1" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_5_2" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_5_3" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="for-deck" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -538,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E22"/>
+  <dimension ref="A2:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -968,35 +969,62 @@
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Table 5.3</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>Table_5_3</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>Chapter V (Paragraph 318 / Image 19)</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Evaluation Dimension 3: Generalizability and Cross-Airport Transfer Performance</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>Zero-shot cross-airport transfer (EWR -&gt; LGA); Model 1 decisive winner, Model 3 fails transfer target.</t>
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Slide 22 Deck Table</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>for-deck</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Defense Presentation (Slide 22)</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>Master Performance Evaluation Across Robustness, Resilience, and Generalizability</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="inlineStr">
+        <is>
+          <t>Certified Slide 22 defense deck summary table comparing Baseline Control, Model 1, Model 2, and Model 3 across all three core evaluation dimensions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Note. This workbook contains a 1-to-1 mapping of all tables embedded within the final thesis manuscript (Thesisv3.docx). Click any tab name to navigate directly to the table.</t>
         </is>
@@ -1019,6 +1047,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3318,6 +3347,395 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>← Return to Table of Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Slide 22 Presentation Table</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>Operational Evaluation Across Robustness, Resilience, and Generalizability (Slide 22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1"/>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Evaluation Dimension</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Operational Regime &amp; Metric</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Academic Target</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Baseline Control</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Model 1 (Deterministic)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Model 2 (Machine Learning)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Model 3 (Dynamic Hybrid)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 1: Robustness</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Routine On-Time Ops (MASE_routine)</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>&lt; 0.700</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>1.000 (Baseline)</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>0.945 (Fails Target)</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>0.680–0.700 (Target Met)</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>0.662 (Target Met / Lowest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 1: Robustness</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Routine Absolute Error (RMSE_routine)</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>253.6 pax/hr</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>313.4 pax/hr</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>273.5 pax/hr</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>222.1 pax/hr (Lowest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 2: Resilience</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Severe IROPS Error Multiplier (R_MASE)</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>≈ 1.00</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>1.000 (Reference)</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>1.32 (Blind to Delays)</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>2.14 (Fragile Collapse)</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>1.05 (Target Met / Winner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 2: Resilience</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Severe Disruption Error (MASE_shock)</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Lowest</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>1.082</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>0.812</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>0.694 (Target Met / Winner)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 2: Resilience</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Time-to-Recovery (TTR, hours)</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>&lt; 4.0h</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>8.4h (Static Reference)</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>7.8h</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>5.4h</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>2.8h (Target Met / Fastest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 3: Generalizability</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Zero-Shot Transfer Ratio (EWR → LGA RTR)</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>≈ 1.00</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>1.00 (Reference)</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>1.04 (Target Met / Winner)</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>1.08 (Passes Target)</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="inlineStr">
+        <is>
+          <t>1.19 (Failed Target)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Dimension 3: Generalizability</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Transfer Error Degradation (ΔRMSE)</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>≤ 10.0%</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>0.0% (Reference)</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>+4.2% (Target Met / Winner)</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>+7.9% (Passes Target)</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>+19.0% (Failed Target)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Dimension 3: Generalizability</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Transfer Relative Error Degradation (ΔMASE)</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>≤ 10.0%</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>0.0% (Reference)</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>+4.0% (Target Met / Winner)</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>+8.3% (Passes Target)</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>+21.5% (Failed Target)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="8" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Note. Reconstructed presentation table for Slide 22 of Master-Thesis-Defense-final.pptx, fully synchronized with certified thesis metrics. Baseline Control: 24h daily persistence benchmark (MASE = 1.000). Model 1: Deterministic flight schedule convolution (t+1, t+2, t+3 show-up curves). Model 2: Supervised machine learning regressor (24 operational features). Model 3: Dynamic two-stage hybrid model (schedule + live 1-step error innovation feedback). Asymmetric Trade-Offs (H1) confirmed: Model 3 achieves lowest routine RMSE (222.1 pax/hr) and decisive shock resilience (R_MASE = 1.05, TTR = 2.8h); Model 2 achieves routine Pareto efficiency (MASE = 0.680–0.700, zero feedback compute latency); Model 1 achieves decisive zero-shot spatial transferability (RTR = 1.04, ΔRMSE = +4.2%, ΔMASE = +4.0%), while Model 3 decisively fails cross-airport transfer (RTR = 1.19, ΔMASE = +21.5%) due to decision tree terminal geometry overfitting.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A1" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>